<commit_message>
fix: generate Excel-compatible assessment exports
</commit_message>
<xml_diff>
--- a/defaults/agentic-potential-assessment/KI-Potentiale.agentic.v1.xlsx
+++ b/defaults/agentic-potential-assessment/KI-Potentiale.agentic.v1.xlsx
@@ -7,7 +7,7 @@
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Agentische Bewertung" sheetId="1" r:id="rId11"/>
+    <sheet name="Agentische Bewertung" sheetId="6" r:id="rId11"/>
     <sheet name="KI-Kernnutzen" sheetId="3" r:id="rId1"/>
     <sheet name="Kriterien Volltext" sheetId="2" r:id="rId2"/>
     <sheet name="Kriterien Kurz" sheetId="1" r:id="rId3"/>
@@ -2067,6 +2067,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2245,10 +2246,10 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A5:J5"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <autoFilter ref="A5:J5"/>
   <printOptions gridLines="0"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>

</xml_diff>